<commit_message>
Full registry refresh Sep 2026: 155/158 active
- Re-fetched 62 parent datasets (NSO live check, MongolBank to Sep 7, MRPAM July)
- Table switches: labor-participation (018V1_10), salary (name-keyed wages),
  air-pollution (V3 SO2-only); livestock-total v3 restores type breakdown
- Deprecate unemployment-by-sex, hospital-beds-by-type, hospital-bed-density
- Regenerate charts, MDX, thumbnails; validation clean
</commit_message>
<xml_diff>
--- a/data.mn/public/datasets/air-pollution-concentration.xlsx
+++ b/data.mn/public/datasets/air-pollution-concentration.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Data" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -413,8 +413,12 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C207"/>
+  <dimension ref="A1:B297"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="9" customWidth="1" min="1" max="1"/>
+    <col width="8" customWidth="1" min="2" max="2"/>
+  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" t="inlineStr">
@@ -424,2653 +428,2968 @@
       </c>
       <c r="B1" t="inlineStr">
         <is>
-          <t>PM10</t>
-        </is>
-      </c>
-      <c r="C1" t="inlineStr">
-        <is>
-          <t>PM2.5</t>
+          <t>SO2</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>2008-12</t>
+          <t>2002-01</t>
         </is>
       </c>
       <c r="B2" t="n">
-        <v>0.58</v>
-      </c>
-      <c r="C2" t="inlineStr"/>
+        <v>0.0267</v>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>2009-01</t>
+          <t>2002-02</t>
         </is>
       </c>
       <c r="B3" t="n">
-        <v>0.512</v>
-      </c>
-      <c r="C3" t="inlineStr"/>
+        <v>0.0193</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>2009-02</t>
+          <t>2002-03</t>
         </is>
       </c>
       <c r="B4" t="n">
-        <v>0.076</v>
-      </c>
-      <c r="C4" t="inlineStr"/>
+        <v>0.0137</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>2009-03</t>
+          <t>2002-04</t>
         </is>
       </c>
       <c r="B5" t="n">
-        <v>0.07199999999999999</v>
-      </c>
-      <c r="C5" t="inlineStr"/>
+        <v>0.008</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>2009-05</t>
+          <t>2002-05</t>
         </is>
       </c>
       <c r="B6" t="n">
-        <v>0.079</v>
-      </c>
-      <c r="C6" t="inlineStr"/>
+        <v>0.0037</v>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>2009-06</t>
+          <t>2002-06</t>
         </is>
       </c>
       <c r="B7" t="n">
-        <v>0.0383</v>
-      </c>
-      <c r="C7" t="inlineStr"/>
+        <v>0.003</v>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>2009-07</t>
+          <t>2002-07</t>
         </is>
       </c>
       <c r="B8" t="n">
-        <v>0.023</v>
-      </c>
-      <c r="C8" t="inlineStr"/>
+        <v>0.0027</v>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>2009-08</t>
+          <t>2002-08</t>
         </is>
       </c>
       <c r="B9" t="n">
-        <v>0.0225</v>
-      </c>
-      <c r="C9" t="inlineStr"/>
+        <v>0.004</v>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>2009-09</t>
+          <t>2002-09</t>
         </is>
       </c>
       <c r="B10" t="n">
-        <v>0.06900000000000001</v>
-      </c>
-      <c r="C10" t="inlineStr"/>
+        <v>0.004</v>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>2009-10</t>
+          <t>2002-10</t>
         </is>
       </c>
       <c r="B11" t="n">
-        <v>0.098</v>
-      </c>
-      <c r="C11" t="inlineStr"/>
+        <v>0.0047</v>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>2009-11</t>
+          <t>2002-11</t>
         </is>
       </c>
       <c r="B12" t="n">
-        <v>0.2</v>
-      </c>
-      <c r="C12" t="inlineStr"/>
+        <v>0.013</v>
+      </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>2009-12</t>
+          <t>2002-12</t>
         </is>
       </c>
       <c r="B13" t="n">
-        <v>0.3202</v>
-      </c>
-      <c r="C13" t="inlineStr"/>
+        <v>0.0277</v>
+      </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>2010-01</t>
+          <t>2003-01</t>
         </is>
       </c>
       <c r="B14" t="n">
-        <v>0.2667</v>
-      </c>
-      <c r="C14" t="inlineStr"/>
+        <v>0.022</v>
+      </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>2010-02</t>
+          <t>2003-02</t>
         </is>
       </c>
       <c r="B15" t="n">
-        <v>0.1937</v>
-      </c>
-      <c r="C15" t="inlineStr"/>
+        <v>0.016</v>
+      </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>2010-03</t>
+          <t>2003-03</t>
         </is>
       </c>
       <c r="B16" t="n">
-        <v>0.153</v>
-      </c>
-      <c r="C16" t="inlineStr"/>
+        <v>0.014</v>
+      </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>2010-04</t>
+          <t>2003-04</t>
         </is>
       </c>
       <c r="B17" t="n">
-        <v>0.0597</v>
-      </c>
-      <c r="C17" t="inlineStr"/>
+        <v>0.0083</v>
+      </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>2010-05</t>
+          <t>2003-05</t>
         </is>
       </c>
       <c r="B18" t="n">
-        <v>0.0453</v>
-      </c>
-      <c r="C18" t="inlineStr"/>
+        <v>0.0053</v>
+      </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>2010-06</t>
+          <t>2003-06</t>
         </is>
       </c>
       <c r="B19" t="n">
-        <v>0.037</v>
-      </c>
-      <c r="C19" t="inlineStr"/>
+        <v>0.0047</v>
+      </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>2010-07</t>
+          <t>2003-07</t>
         </is>
       </c>
       <c r="B20" t="n">
-        <v>0.052</v>
-      </c>
-      <c r="C20" t="n">
-        <v>0.0235</v>
+        <v>0.003</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>2010-08</t>
+          <t>2003-08</t>
         </is>
       </c>
       <c r="B21" t="n">
-        <v>0.09080000000000001</v>
-      </c>
-      <c r="C21" t="inlineStr"/>
+        <v>0.0027</v>
+      </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>2010-09</t>
+          <t>2003-09</t>
         </is>
       </c>
       <c r="B22" t="n">
-        <v>0.1258</v>
-      </c>
-      <c r="C22" t="n">
-        <v>0.0375</v>
+        <v>0.0025</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>2010-10</t>
+          <t>2003-10</t>
         </is>
       </c>
       <c r="B23" t="n">
-        <v>0.1565</v>
-      </c>
-      <c r="C23" t="n">
-        <v>0.0595</v>
+        <v>0.0075</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>2010-11</t>
+          <t>2003-11</t>
         </is>
       </c>
       <c r="B24" t="n">
-        <v>0.221</v>
-      </c>
-      <c r="C24" t="n">
-        <v>0.144</v>
+        <v>0.02</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>2010-12</t>
+          <t>2003-12</t>
         </is>
       </c>
       <c r="B25" t="n">
-        <v>0.3846</v>
-      </c>
-      <c r="C25" t="n">
-        <v>0.4</v>
+        <v>0.0407</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>2011-01</t>
+          <t>2004-01</t>
         </is>
       </c>
       <c r="B26" t="n">
-        <v>0.436</v>
-      </c>
-      <c r="C26" t="n">
-        <v>0.459</v>
+        <v>0.0395</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>2011-02</t>
+          <t>2004-02</t>
         </is>
       </c>
       <c r="B27" t="n">
-        <v>0.3517</v>
-      </c>
-      <c r="C27" t="n">
-        <v>0.27</v>
+        <v>0.028</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>2011-03</t>
+          <t>2004-03</t>
         </is>
       </c>
       <c r="B28" t="n">
-        <v>0.1755</v>
-      </c>
-      <c r="C28" t="n">
-        <v>0.127</v>
+        <v>0.0157</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>2011-04</t>
+          <t>2004-04</t>
         </is>
       </c>
       <c r="B29" t="n">
-        <v>0.202</v>
-      </c>
-      <c r="C29" t="n">
-        <v>0.051</v>
+        <v>0.0072</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>2011-05</t>
+          <t>2004-05</t>
         </is>
       </c>
       <c r="B30" t="n">
-        <v>0.146</v>
-      </c>
-      <c r="C30" t="n">
-        <v>0.042</v>
+        <v>0.0038</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>2011-06</t>
+          <t>2004-06</t>
         </is>
       </c>
       <c r="B31" t="n">
-        <v>0.1123</v>
-      </c>
-      <c r="C31" t="n">
-        <v>0.0445</v>
+        <v>0.0032</v>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>2011-07</t>
+          <t>2004-07</t>
         </is>
       </c>
       <c r="B32" t="n">
-        <v>0.1187</v>
-      </c>
-      <c r="C32" t="n">
-        <v>0.0555</v>
+        <v>0.0037</v>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>2011-08</t>
+          <t>2004-08</t>
         </is>
       </c>
       <c r="B33" t="n">
-        <v>0.129</v>
-      </c>
-      <c r="C33" t="n">
-        <v>0.044</v>
+        <v>0.0037</v>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>2011-09</t>
+          <t>2004-09</t>
         </is>
       </c>
       <c r="B34" t="n">
-        <v>0.1478</v>
-      </c>
-      <c r="C34" t="n">
-        <v>0.0395</v>
+        <v>0.0047</v>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>2011-10</t>
+          <t>2004-10</t>
         </is>
       </c>
       <c r="B35" t="n">
-        <v>0.156</v>
-      </c>
-      <c r="C35" t="n">
-        <v>0.0625</v>
+        <v>0.0105</v>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>2011-11</t>
+          <t>2004-11</t>
         </is>
       </c>
       <c r="B36" t="n">
-        <v>0.2838</v>
-      </c>
-      <c r="C36" t="n">
-        <v>0.119</v>
+        <v>0.0233</v>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>2011-12</t>
+          <t>2004-12</t>
         </is>
       </c>
       <c r="B37" t="n">
-        <v>0.7945</v>
-      </c>
-      <c r="C37" t="n">
-        <v>0.318</v>
+        <v>0.027</v>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>2012-01</t>
+          <t>2005-01</t>
         </is>
       </c>
       <c r="B38" t="n">
-        <v>0.8362000000000001</v>
-      </c>
-      <c r="C38" t="n">
-        <v>0.27</v>
+        <v>0.0373</v>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>2012-02</t>
+          <t>2005-02</t>
         </is>
       </c>
       <c r="B39" t="n">
-        <v>0.4318</v>
-      </c>
-      <c r="C39" t="n">
-        <v>0.153</v>
+        <v>0.029</v>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>2012-03</t>
+          <t>2005-03</t>
         </is>
       </c>
       <c r="B40" t="n">
-        <v>0.2094</v>
-      </c>
-      <c r="C40" t="n">
-        <v>0.082</v>
+        <v>0.0162</v>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>2012-04</t>
+          <t>2005-04</t>
         </is>
       </c>
       <c r="B41" t="n">
-        <v>0.271</v>
-      </c>
-      <c r="C41" t="n">
-        <v>0.036</v>
+        <v>0.008800000000000001</v>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>2012-05</t>
+          <t>2005-05</t>
         </is>
       </c>
       <c r="B42" t="n">
-        <v>0.3025</v>
-      </c>
-      <c r="C42" t="n">
-        <v>0.035</v>
+        <v>0.0052</v>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>2012-06</t>
+          <t>2005-06</t>
         </is>
       </c>
       <c r="B43" t="n">
-        <v>0.104</v>
-      </c>
-      <c r="C43" t="n">
-        <v>0.035</v>
+        <v>0.0028</v>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>2012-07</t>
+          <t>2005-07</t>
         </is>
       </c>
       <c r="B44" t="n">
-        <v>0.1088</v>
-      </c>
-      <c r="C44" t="n">
-        <v>0.035</v>
+        <v>0.0028</v>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>2012-08</t>
+          <t>2005-08</t>
         </is>
       </c>
       <c r="B45" t="n">
-        <v>0.134</v>
-      </c>
-      <c r="C45" t="n">
-        <v>0.039</v>
+        <v>0.003</v>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>2012-09</t>
+          <t>2005-09</t>
         </is>
       </c>
       <c r="B46" t="n">
-        <v>0.1347</v>
-      </c>
-      <c r="C46" t="n">
-        <v>0.043</v>
+        <v>0.0043</v>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>2012-10</t>
+          <t>2005-10</t>
         </is>
       </c>
       <c r="B47" t="n">
-        <v>0.1595</v>
-      </c>
-      <c r="C47" t="n">
-        <v>0.014</v>
+        <v>0.008200000000000001</v>
       </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>2012-11</t>
+          <t>2005-11</t>
         </is>
       </c>
       <c r="B48" t="n">
-        <v>0.254</v>
-      </c>
-      <c r="C48" t="n">
-        <v>0.133</v>
+        <v>0.0145</v>
       </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>2012-12</t>
+          <t>2005-12</t>
         </is>
       </c>
       <c r="B49" t="n">
-        <v>0.5377</v>
-      </c>
-      <c r="C49" t="n">
-        <v>0.224</v>
+        <v>0.0207</v>
       </c>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>2013-01</t>
+          <t>2006-01</t>
         </is>
       </c>
       <c r="B50" t="n">
-        <v>0.6858</v>
-      </c>
-      <c r="C50" t="n">
-        <v>0.622</v>
+        <v>0.027</v>
       </c>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>2013-02</t>
+          <t>2006-02</t>
         </is>
       </c>
       <c r="B51" t="n">
-        <v>0.2576</v>
-      </c>
-      <c r="C51" t="n">
-        <v>0.15</v>
+        <v>0.0207</v>
       </c>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>2013-03</t>
+          <t>2006-03</t>
         </is>
       </c>
       <c r="B52" t="n">
-        <v>0.1558</v>
-      </c>
-      <c r="C52" t="n">
-        <v>0.068</v>
+        <v>0.0135</v>
       </c>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>2013-04</t>
+          <t>2006-04</t>
         </is>
       </c>
       <c r="B53" t="n">
-        <v>0.1266</v>
-      </c>
-      <c r="C53" t="n">
-        <v>0.035</v>
+        <v>0.008999999999999999</v>
       </c>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>2013-05</t>
+          <t>2006-05</t>
         </is>
       </c>
       <c r="B54" t="n">
-        <v>0.128</v>
-      </c>
-      <c r="C54" t="n">
-        <v>0.035</v>
+        <v>0.0068</v>
       </c>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>2013-06</t>
+          <t>2006-06</t>
         </is>
       </c>
       <c r="B55" t="n">
-        <v>0.09719999999999999</v>
-      </c>
-      <c r="C55" t="n">
-        <v>0.0305</v>
+        <v>0.0018</v>
       </c>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>2013-07</t>
+          <t>2006-07</t>
         </is>
       </c>
       <c r="B56" t="n">
-        <v>0.094</v>
-      </c>
-      <c r="C56" t="n">
-        <v>0.0335</v>
+        <v>0.0018</v>
       </c>
     </row>
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>2013-08</t>
+          <t>2006-08</t>
         </is>
       </c>
       <c r="B57" t="n">
-        <v>0.1096</v>
-      </c>
-      <c r="C57" t="n">
-        <v>0.0415</v>
+        <v>0.003</v>
       </c>
     </row>
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>2013-09</t>
+          <t>2006-09</t>
         </is>
       </c>
       <c r="B58" t="n">
-        <v>0.1266</v>
-      </c>
-      <c r="C58" t="n">
-        <v>0.0315</v>
+        <v>0.0038</v>
       </c>
     </row>
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>2013-10</t>
+          <t>2006-10</t>
         </is>
       </c>
       <c r="B59" t="n">
-        <v>0.1738</v>
-      </c>
-      <c r="C59" t="n">
-        <v>0.05</v>
+        <v>0.0118</v>
       </c>
     </row>
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>2013-11</t>
+          <t>2006-11</t>
         </is>
       </c>
       <c r="B60" t="n">
-        <v>0.2414</v>
-      </c>
-      <c r="C60" t="n">
-        <v>0.1135</v>
+        <v>0.022</v>
       </c>
     </row>
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>2013-12</t>
+          <t>2006-12</t>
         </is>
       </c>
       <c r="B61" t="n">
-        <v>0.3838</v>
-      </c>
-      <c r="C61" t="n">
-        <v>0.1855</v>
+        <v>0.031</v>
       </c>
     </row>
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>2014-01</t>
+          <t>2007-01</t>
         </is>
       </c>
       <c r="B62" t="n">
-        <v>0.3838</v>
-      </c>
-      <c r="C62" t="n">
-        <v>0.166</v>
+        <v>0.034</v>
       </c>
     </row>
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>2014-02</t>
+          <t>2007-02</t>
         </is>
       </c>
       <c r="B63" t="n">
-        <v>0.2586</v>
-      </c>
-      <c r="C63" t="n">
-        <v>0.109</v>
+        <v>0.024</v>
       </c>
     </row>
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t>2014-03</t>
+          <t>2007-03</t>
         </is>
       </c>
       <c r="B64" t="n">
-        <v>0.1732</v>
-      </c>
-      <c r="C64" t="n">
-        <v>0.0555</v>
+        <v>0.0185</v>
       </c>
     </row>
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>2014-04</t>
+          <t>2007-04</t>
         </is>
       </c>
       <c r="B65" t="n">
-        <v>0.1547</v>
-      </c>
-      <c r="C65" t="n">
-        <v>0.033</v>
+        <v>0.0072</v>
       </c>
     </row>
     <row r="66">
       <c r="A66" t="inlineStr">
         <is>
-          <t>2014-05</t>
+          <t>2007-05</t>
         </is>
       </c>
       <c r="B66" t="n">
-        <v>0.1057</v>
-      </c>
-      <c r="C66" t="n">
-        <v>0.0215</v>
+        <v>0.0042</v>
       </c>
     </row>
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>2014-06</t>
+          <t>2007-06</t>
         </is>
       </c>
       <c r="B67" t="n">
-        <v>0.1186</v>
-      </c>
-      <c r="C67" t="n">
-        <v>0.0165</v>
+        <v>0.0042</v>
       </c>
     </row>
     <row r="68">
       <c r="A68" t="inlineStr">
         <is>
-          <t>2014-07</t>
+          <t>2007-07</t>
         </is>
       </c>
       <c r="B68" t="n">
-        <v>0.097</v>
-      </c>
-      <c r="C68" t="n">
-        <v>0.022</v>
+        <v>0.0038</v>
       </c>
     </row>
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t>2014-08</t>
+          <t>2007-08</t>
         </is>
       </c>
       <c r="B69" t="n">
-        <v>0.1258</v>
-      </c>
-      <c r="C69" t="n">
-        <v>0.0215</v>
+        <v>0.0015</v>
       </c>
     </row>
     <row r="70">
       <c r="A70" t="inlineStr">
         <is>
-          <t>2014-09</t>
+          <t>2007-09</t>
         </is>
       </c>
       <c r="B70" t="n">
-        <v>0.1446</v>
-      </c>
-      <c r="C70" t="n">
-        <v>0.035</v>
+        <v>0.0025</v>
       </c>
     </row>
     <row r="71">
       <c r="A71" t="inlineStr">
         <is>
-          <t>2014-10</t>
+          <t>2007-10</t>
         </is>
       </c>
       <c r="B71" t="n">
-        <v>0.1708</v>
-      </c>
-      <c r="C71" t="n">
-        <v>0.0535</v>
+        <v>0.0062</v>
       </c>
     </row>
     <row r="72">
       <c r="A72" t="inlineStr">
         <is>
-          <t>2014-11</t>
+          <t>2007-11</t>
         </is>
       </c>
       <c r="B72" t="n">
-        <v>0.2048</v>
-      </c>
-      <c r="C72" t="n">
-        <v>0.0895</v>
+        <v>0.01</v>
       </c>
     </row>
     <row r="73">
       <c r="A73" t="inlineStr">
         <is>
-          <t>2014-12</t>
+          <t>2007-12</t>
         </is>
       </c>
       <c r="B73" t="n">
-        <v>0.2366</v>
-      </c>
-      <c r="C73" t="n">
-        <v>0.1475</v>
+        <v>0.0173</v>
       </c>
     </row>
     <row r="74">
       <c r="A74" t="inlineStr">
         <is>
-          <t>2015-01</t>
+          <t>2008-01</t>
         </is>
       </c>
       <c r="B74" t="n">
-        <v>0.2277</v>
-      </c>
-      <c r="C74" t="n">
-        <v>0.1852</v>
+        <v>0.0262</v>
       </c>
     </row>
     <row r="75">
       <c r="A75" t="inlineStr">
         <is>
-          <t>2015-02</t>
+          <t>2008-02</t>
         </is>
       </c>
       <c r="B75" t="n">
-        <v>0.208</v>
-      </c>
-      <c r="C75" t="n">
-        <v>0.1203</v>
+        <v>0.0258</v>
       </c>
     </row>
     <row r="76">
       <c r="A76" t="inlineStr">
         <is>
-          <t>2015-03</t>
+          <t>2008-03</t>
         </is>
       </c>
       <c r="B76" t="n">
-        <v>0.1427</v>
-      </c>
-      <c r="C76" t="n">
-        <v>0.08</v>
+        <v>0.0162</v>
       </c>
     </row>
     <row r="77">
       <c r="A77" t="inlineStr">
         <is>
-          <t>2015-04</t>
+          <t>2008-04</t>
         </is>
       </c>
       <c r="B77" t="n">
-        <v>0.136</v>
-      </c>
-      <c r="C77" t="n">
-        <v>0.0487</v>
+        <v>0.008999999999999999</v>
       </c>
     </row>
     <row r="78">
       <c r="A78" t="inlineStr">
         <is>
-          <t>2015-05</t>
+          <t>2008-05</t>
         </is>
       </c>
       <c r="B78" t="n">
-        <v>0.1043</v>
-      </c>
-      <c r="C78" t="n">
-        <v>0.0315</v>
+        <v>0.0033</v>
       </c>
     </row>
     <row r="79">
       <c r="A79" t="inlineStr">
         <is>
-          <t>2015-06</t>
+          <t>2008-06</t>
         </is>
       </c>
       <c r="B79" t="n">
-        <v>0.0953</v>
-      </c>
-      <c r="C79" t="n">
-        <v>0.0255</v>
+        <v>0.0033</v>
       </c>
     </row>
     <row r="80">
       <c r="A80" t="inlineStr">
         <is>
-          <t>2015-07</t>
+          <t>2008-07</t>
         </is>
       </c>
       <c r="B80" t="n">
-        <v>0.074</v>
-      </c>
-      <c r="C80" t="n">
-        <v>0.022</v>
+        <v>0.0005</v>
       </c>
     </row>
     <row r="81">
       <c r="A81" t="inlineStr">
         <is>
-          <t>2015-08</t>
+          <t>2008-08</t>
         </is>
       </c>
       <c r="B81" t="n">
-        <v>0.08699999999999999</v>
-      </c>
-      <c r="C81" t="n">
-        <v>0.0238</v>
+        <v>0.002</v>
       </c>
     </row>
     <row r="82">
       <c r="A82" t="inlineStr">
         <is>
-          <t>2015-09</t>
+          <t>2008-09</t>
         </is>
       </c>
       <c r="B82" t="n">
-        <v>0.0847</v>
-      </c>
-      <c r="C82" t="n">
-        <v>0.0272</v>
+        <v>0.003</v>
       </c>
     </row>
     <row r="83">
       <c r="A83" t="inlineStr">
         <is>
-          <t>2015-10</t>
+          <t>2008-10</t>
         </is>
       </c>
       <c r="B83" t="n">
-        <v>0.1393</v>
-      </c>
-      <c r="C83" t="n">
-        <v>0.0583</v>
+        <v>0.007</v>
       </c>
     </row>
     <row r="84">
       <c r="A84" t="inlineStr">
         <is>
-          <t>2015-11</t>
+          <t>2008-11</t>
         </is>
       </c>
       <c r="B84" t="n">
-        <v>0.1557</v>
-      </c>
-      <c r="C84" t="n">
-        <v>0.1148</v>
+        <v>0.0305</v>
       </c>
     </row>
     <row r="85">
       <c r="A85" t="inlineStr">
         <is>
-          <t>2015-12</t>
+          <t>2008-12</t>
         </is>
       </c>
       <c r="B85" t="n">
-        <v>0.1811</v>
-      </c>
-      <c r="C85" t="n">
-        <v>0.1612</v>
+        <v>0.0424</v>
       </c>
     </row>
     <row r="86">
       <c r="A86" t="inlineStr">
         <is>
-          <t>2016-01</t>
+          <t>2009-01</t>
         </is>
       </c>
       <c r="B86" t="n">
-        <v>0.2246</v>
-      </c>
-      <c r="C86" t="n">
-        <v>0.1964</v>
+        <v>0.0413</v>
       </c>
     </row>
     <row r="87">
       <c r="A87" t="inlineStr">
         <is>
-          <t>2016-02</t>
+          <t>2009-02</t>
         </is>
       </c>
       <c r="B87" t="n">
-        <v>0.176</v>
-      </c>
-      <c r="C87" t="n">
-        <v>0.1395</v>
+        <v>0.032</v>
       </c>
     </row>
     <row r="88">
       <c r="A88" t="inlineStr">
         <is>
-          <t>2016-03</t>
+          <t>2009-03</t>
         </is>
       </c>
       <c r="B88" t="n">
-        <v>0.1001</v>
-      </c>
-      <c r="C88" t="n">
-        <v>0.0615</v>
+        <v>0.0225</v>
       </c>
     </row>
     <row r="89">
       <c r="A89" t="inlineStr">
         <is>
-          <t>2016-04</t>
+          <t>2009-04</t>
         </is>
       </c>
       <c r="B89" t="n">
-        <v>0.1059</v>
-      </c>
-      <c r="C89" t="n">
-        <v>0.0335</v>
+        <v>0.0113</v>
       </c>
     </row>
     <row r="90">
       <c r="A90" t="inlineStr">
         <is>
-          <t>2016-05</t>
+          <t>2009-05</t>
         </is>
       </c>
       <c r="B90" t="n">
-        <v>0.089</v>
-      </c>
-      <c r="C90" t="n">
-        <v>0.0252</v>
+        <v>0.0043</v>
       </c>
     </row>
     <row r="91">
       <c r="A91" t="inlineStr">
         <is>
-          <t>2016-06</t>
+          <t>2009-06</t>
         </is>
       </c>
       <c r="B91" t="n">
-        <v>0.0725</v>
-      </c>
-      <c r="C91" t="n">
-        <v>0.0237</v>
+        <v>0.0033</v>
       </c>
     </row>
     <row r="92">
       <c r="A92" t="inlineStr">
         <is>
-          <t>2016-07</t>
+          <t>2009-07</t>
         </is>
       </c>
       <c r="B92" t="n">
-        <v>0.0915</v>
-      </c>
-      <c r="C92" t="n">
-        <v>0.035</v>
+        <v>0.001</v>
       </c>
     </row>
     <row r="93">
       <c r="A93" t="inlineStr">
         <is>
-          <t>2016-08</t>
+          <t>2009-08</t>
         </is>
       </c>
       <c r="B93" t="n">
-        <v>0.0639</v>
-      </c>
-      <c r="C93" t="n">
-        <v>0.0143</v>
+        <v>0.0022</v>
       </c>
     </row>
     <row r="94">
       <c r="A94" t="inlineStr">
         <is>
-          <t>2016-09</t>
+          <t>2009-09</t>
         </is>
       </c>
       <c r="B94" t="n">
-        <v>0.0901</v>
-      </c>
-      <c r="C94" t="n">
-        <v>0.0325</v>
+        <v>0.004</v>
       </c>
     </row>
     <row r="95">
       <c r="A95" t="inlineStr">
         <is>
-          <t>2016-10</t>
+          <t>2009-10</t>
         </is>
       </c>
       <c r="B95" t="n">
-        <v>0.1195</v>
-      </c>
-      <c r="C95" t="n">
-        <v>0.0572</v>
+        <v>0.0126</v>
       </c>
     </row>
     <row r="96">
       <c r="A96" t="inlineStr">
         <is>
-          <t>2016-11</t>
+          <t>2009-11</t>
         </is>
       </c>
       <c r="B96" t="n">
-        <v>0.1884</v>
-      </c>
-      <c r="C96" t="n">
-        <v>0.1512</v>
+        <v>0.0428</v>
       </c>
     </row>
     <row r="97">
       <c r="A97" t="inlineStr">
         <is>
-          <t>2016-12</t>
+          <t>2009-12</t>
         </is>
       </c>
       <c r="B97" t="n">
-        <v>0.224</v>
-      </c>
-      <c r="C97" t="n">
-        <v>0.2037</v>
+        <v>0.065</v>
       </c>
     </row>
     <row r="98">
       <c r="A98" t="inlineStr">
         <is>
-          <t>2017-01</t>
+          <t>2010-01</t>
         </is>
       </c>
       <c r="B98" t="n">
-        <v>0.2208</v>
-      </c>
-      <c r="C98" t="n">
-        <v>0.198</v>
+        <v>0.0698</v>
       </c>
     </row>
     <row r="99">
       <c r="A99" t="inlineStr">
         <is>
-          <t>2017-02</t>
+          <t>2010-02</t>
         </is>
       </c>
       <c r="B99" t="n">
-        <v>0.1566</v>
-      </c>
-      <c r="C99" t="n">
-        <v>0.1337</v>
+        <v>0.056</v>
       </c>
     </row>
     <row r="100">
       <c r="A100" t="inlineStr">
         <is>
-          <t>2017-03</t>
+          <t>2010-03</t>
         </is>
       </c>
       <c r="B100" t="n">
-        <v>0.0969</v>
-      </c>
-      <c r="C100" t="n">
-        <v>0.0505</v>
+        <v>0.0302</v>
       </c>
     </row>
     <row r="101">
       <c r="A101" t="inlineStr">
         <is>
-          <t>2017-04</t>
+          <t>2010-04</t>
         </is>
       </c>
       <c r="B101" t="n">
-        <v>0.1289</v>
-      </c>
-      <c r="C101" t="n">
-        <v>0.0435</v>
+        <v>0.0148</v>
       </c>
     </row>
     <row r="102">
       <c r="A102" t="inlineStr">
         <is>
-          <t>2017-05</t>
+          <t>2010-05</t>
         </is>
       </c>
       <c r="B102" t="n">
-        <v>0.1069</v>
-      </c>
-      <c r="C102" t="n">
-        <v>0.0243</v>
+        <v>0.006</v>
       </c>
     </row>
     <row r="103">
       <c r="A103" t="inlineStr">
         <is>
-          <t>2017-06</t>
+          <t>2010-06</t>
         </is>
       </c>
       <c r="B103" t="n">
-        <v>0.09950000000000001</v>
-      </c>
-      <c r="C103" t="n">
-        <v>0.0223</v>
+        <v>0.0023</v>
       </c>
     </row>
     <row r="104">
       <c r="A104" t="inlineStr">
         <is>
-          <t>2017-07</t>
+          <t>2010-07</t>
         </is>
       </c>
       <c r="B104" t="n">
-        <v>0.0771</v>
-      </c>
-      <c r="C104" t="n">
-        <v>0.1037</v>
+        <v>0.0046</v>
       </c>
     </row>
     <row r="105">
       <c r="A105" t="inlineStr">
         <is>
-          <t>2017-08</t>
+          <t>2010-08</t>
         </is>
       </c>
       <c r="B105" t="n">
-        <v>0.0473</v>
-      </c>
-      <c r="C105" t="n">
-        <v>0.0152</v>
+        <v>0.0071</v>
       </c>
     </row>
     <row r="106">
       <c r="A106" t="inlineStr">
         <is>
-          <t>2017-09</t>
+          <t>2010-09</t>
         </is>
       </c>
       <c r="B106" t="n">
-        <v>0.0743</v>
-      </c>
-      <c r="C106" t="n">
-        <v>0.0237</v>
+        <v>0.008399999999999999</v>
       </c>
     </row>
     <row r="107">
       <c r="A107" t="inlineStr">
         <is>
-          <t>2017-10</t>
+          <t>2010-10</t>
         </is>
       </c>
       <c r="B107" t="n">
-        <v>0.1234</v>
-      </c>
-      <c r="C107" t="n">
-        <v>0.0617</v>
+        <v>0.018</v>
       </c>
     </row>
     <row r="108">
       <c r="A108" t="inlineStr">
         <is>
-          <t>2017-11</t>
+          <t>2010-11</t>
         </is>
       </c>
       <c r="B108" t="n">
-        <v>0.1433</v>
-      </c>
-      <c r="C108" t="n">
-        <v>0.116</v>
+        <v>0.0407</v>
       </c>
     </row>
     <row r="109">
       <c r="A109" t="inlineStr">
         <is>
-          <t>2017-12</t>
+          <t>2010-12</t>
         </is>
       </c>
       <c r="B109" t="n">
-        <v>0.2122</v>
-      </c>
-      <c r="C109" t="n">
-        <v>0.1735</v>
+        <v>0.0602</v>
       </c>
     </row>
     <row r="110">
       <c r="A110" t="inlineStr">
         <is>
-          <t>2018-01</t>
+          <t>2011-01</t>
         </is>
       </c>
       <c r="B110" t="n">
-        <v>0.2172</v>
-      </c>
-      <c r="C110" t="n">
-        <v>0.1939</v>
+        <v>0.0617</v>
       </c>
     </row>
     <row r="111">
       <c r="A111" t="inlineStr">
         <is>
-          <t>2018-02</t>
+          <t>2011-02</t>
         </is>
       </c>
       <c r="B111" t="n">
-        <v>0.1759</v>
-      </c>
-      <c r="C111" t="n">
-        <v>0.1416</v>
+        <v>0.06900000000000001</v>
       </c>
     </row>
     <row r="112">
       <c r="A112" t="inlineStr">
         <is>
-          <t>2018-03</t>
+          <t>2011-03</t>
         </is>
       </c>
       <c r="B112" t="n">
-        <v>0.1209</v>
-      </c>
-      <c r="C112" t="n">
-        <v>0.0533</v>
+        <v>0.0413</v>
       </c>
     </row>
     <row r="113">
       <c r="A113" t="inlineStr">
         <is>
-          <t>2018-04</t>
+          <t>2011-04</t>
         </is>
       </c>
       <c r="B113" t="n">
-        <v>0.1032</v>
-      </c>
-      <c r="C113" t="n">
-        <v>0.029</v>
+        <v>0.0242</v>
       </c>
     </row>
     <row r="114">
       <c r="A114" t="inlineStr">
         <is>
-          <t>2018-05</t>
+          <t>2011-05</t>
         </is>
       </c>
       <c r="B114" t="n">
-        <v>0.1204</v>
-      </c>
-      <c r="C114" t="n">
-        <v>0.0201</v>
+        <v>0.0123</v>
       </c>
     </row>
     <row r="115">
       <c r="A115" t="inlineStr">
         <is>
-          <t>2018-06</t>
+          <t>2011-06</t>
         </is>
       </c>
       <c r="B115" t="n">
-        <v>0.07489999999999999</v>
-      </c>
-      <c r="C115" t="n">
-        <v>0.0159</v>
+        <v>0.008200000000000001</v>
       </c>
     </row>
     <row r="116">
       <c r="A116" t="inlineStr">
         <is>
-          <t>2018-07</t>
+          <t>2011-07</t>
         </is>
       </c>
       <c r="B116" t="n">
-        <v>0.0402</v>
-      </c>
-      <c r="C116" t="n">
-        <v>0.0124</v>
+        <v>0.006</v>
       </c>
     </row>
     <row r="117">
       <c r="A117" t="inlineStr">
         <is>
-          <t>2018-08</t>
+          <t>2011-08</t>
         </is>
       </c>
       <c r="B117" t="n">
-        <v>0.0509</v>
-      </c>
-      <c r="C117" t="n">
-        <v>0.0153</v>
+        <v>0.0055</v>
       </c>
     </row>
     <row r="118">
       <c r="A118" t="inlineStr">
         <is>
-          <t>2018-09</t>
+          <t>2011-09</t>
         </is>
       </c>
       <c r="B118" t="n">
-        <v>0.0728</v>
-      </c>
-      <c r="C118" t="n">
-        <v>0.0223</v>
+        <v>0.0076</v>
       </c>
     </row>
     <row r="119">
       <c r="A119" t="inlineStr">
         <is>
-          <t>2018-10</t>
+          <t>2011-10</t>
         </is>
       </c>
       <c r="B119" t="n">
-        <v>0.1284</v>
-      </c>
-      <c r="C119" t="n">
-        <v>0.0491</v>
+        <v>0.0176</v>
       </c>
     </row>
     <row r="120">
       <c r="A120" t="inlineStr">
         <is>
-          <t>2018-11</t>
+          <t>2011-11</t>
         </is>
       </c>
       <c r="B120" t="n">
-        <v>0.2001</v>
-      </c>
-      <c r="C120" t="n">
-        <v>0.1054</v>
+        <v>0.0485</v>
       </c>
     </row>
     <row r="121">
       <c r="A121" t="inlineStr">
         <is>
-          <t>2018-12</t>
+          <t>2011-12</t>
         </is>
       </c>
       <c r="B121" t="n">
-        <v>0.2259</v>
-      </c>
-      <c r="C121" t="n">
-        <v>0.1766</v>
+        <v>0.1112</v>
       </c>
     </row>
     <row r="122">
       <c r="A122" t="inlineStr">
         <is>
-          <t>2019-01</t>
+          <t>2012-01</t>
         </is>
       </c>
       <c r="B122" t="n">
-        <v>0.2391</v>
-      </c>
-      <c r="C122" t="n">
-        <v>0.1949</v>
+        <v>0.1004</v>
       </c>
     </row>
     <row r="123">
       <c r="A123" t="inlineStr">
         <is>
-          <t>2019-02</t>
+          <t>2012-02</t>
         </is>
       </c>
       <c r="B123" t="n">
-        <v>0.1764</v>
-      </c>
-      <c r="C123" t="n">
-        <v>0.1124</v>
+        <v>0.07340000000000001</v>
       </c>
     </row>
     <row r="124">
       <c r="A124" t="inlineStr">
         <is>
-          <t>2019-03</t>
+          <t>2012-03</t>
         </is>
       </c>
       <c r="B124" t="n">
-        <v>0.1401</v>
-      </c>
-      <c r="C124" t="n">
-        <v>0.0599</v>
+        <v>0.0379</v>
       </c>
     </row>
     <row r="125">
       <c r="A125" t="inlineStr">
         <is>
-          <t>2019-04</t>
+          <t>2012-04</t>
         </is>
       </c>
       <c r="B125" t="n">
-        <v>0.1076</v>
-      </c>
-      <c r="C125" t="n">
-        <v>0.0321</v>
+        <v>0.0158</v>
       </c>
     </row>
     <row r="126">
       <c r="A126" t="inlineStr">
         <is>
-          <t>2019-05</t>
+          <t>2012-05</t>
         </is>
       </c>
       <c r="B126" t="n">
-        <v>0.083</v>
-      </c>
-      <c r="C126" t="n">
-        <v>0.0208</v>
+        <v>0.009299999999999999</v>
       </c>
     </row>
     <row r="127">
       <c r="A127" t="inlineStr">
         <is>
-          <t>2019-06</t>
+          <t>2012-06</t>
         </is>
       </c>
       <c r="B127" t="n">
-        <v>0.0636</v>
-      </c>
-      <c r="C127" t="n">
-        <v>0.013</v>
+        <v>0.0063</v>
       </c>
     </row>
     <row r="128">
       <c r="A128" t="inlineStr">
         <is>
-          <t>2019-07</t>
+          <t>2012-07</t>
         </is>
       </c>
       <c r="B128" t="n">
-        <v>0.0494</v>
-      </c>
-      <c r="C128" t="n">
-        <v>0.0177</v>
+        <v>0.0045</v>
       </c>
     </row>
     <row r="129">
       <c r="A129" t="inlineStr">
         <is>
-          <t>2019-08</t>
+          <t>2012-08</t>
         </is>
       </c>
       <c r="B129" t="n">
-        <v>0.06</v>
-      </c>
-      <c r="C129" t="n">
-        <v>0.0144</v>
+        <v>0.0033</v>
       </c>
     </row>
     <row r="130">
       <c r="A130" t="inlineStr">
         <is>
-          <t>2019-09</t>
+          <t>2012-09</t>
         </is>
       </c>
       <c r="B130" t="n">
-        <v>0.1054</v>
-      </c>
-      <c r="C130" t="n">
-        <v>0.0223</v>
+        <v>0.0047</v>
       </c>
     </row>
     <row r="131">
       <c r="A131" t="inlineStr">
         <is>
-          <t>2019-10</t>
+          <t>2012-10</t>
         </is>
       </c>
       <c r="B131" t="n">
-        <v>0.1179</v>
-      </c>
-      <c r="C131" t="n">
-        <v>0.0393</v>
+        <v>0.0165</v>
       </c>
     </row>
     <row r="132">
       <c r="A132" t="inlineStr">
         <is>
-          <t>2019-11</t>
+          <t>2012-11</t>
         </is>
       </c>
       <c r="B132" t="n">
-        <v>0.1208</v>
-      </c>
-      <c r="C132" t="n">
-        <v>0.0608</v>
+        <v>0.036</v>
       </c>
     </row>
     <row r="133">
       <c r="A133" t="inlineStr">
         <is>
-          <t>2019-12</t>
+          <t>2012-12</t>
         </is>
       </c>
       <c r="B133" t="n">
-        <v>0.1378</v>
-      </c>
-      <c r="C133" t="n">
-        <v>0.1125</v>
+        <v>0.0698</v>
       </c>
     </row>
     <row r="134">
       <c r="A134" t="inlineStr">
         <is>
-          <t>2020-01</t>
+          <t>2013-01</t>
         </is>
       </c>
       <c r="B134" t="n">
-        <v>0.1285</v>
-      </c>
-      <c r="C134" t="n">
-        <v>0.1036</v>
+        <v>0.09030000000000001</v>
       </c>
     </row>
     <row r="135">
       <c r="A135" t="inlineStr">
         <is>
-          <t>2020-02</t>
+          <t>2013-02</t>
         </is>
       </c>
       <c r="B135" t="n">
-        <v>0.09719999999999999</v>
-      </c>
-      <c r="C135" t="n">
-        <v>0.0682</v>
+        <v>0.0563</v>
       </c>
     </row>
     <row r="136">
       <c r="A136" t="inlineStr">
         <is>
-          <t>2020-03</t>
+          <t>2013-03</t>
         </is>
       </c>
       <c r="B136" t="n">
-        <v>0.07530000000000001</v>
-      </c>
-      <c r="C136" t="n">
-        <v>0.0351</v>
+        <v>0.0233</v>
       </c>
     </row>
     <row r="137">
       <c r="A137" t="inlineStr">
         <is>
-          <t>2020-04</t>
+          <t>2013-04</t>
         </is>
       </c>
       <c r="B137" t="n">
-        <v>0.0993</v>
-      </c>
-      <c r="C137" t="n">
-        <v>0.0295</v>
+        <v>0.0105</v>
       </c>
     </row>
     <row r="138">
       <c r="A138" t="inlineStr">
         <is>
-          <t>2020-05</t>
+          <t>2013-05</t>
         </is>
       </c>
       <c r="B138" t="n">
-        <v>0.0717</v>
-      </c>
-      <c r="C138" t="n">
-        <v>0.0178</v>
+        <v>0.0067</v>
       </c>
     </row>
     <row r="139">
       <c r="A139" t="inlineStr">
         <is>
-          <t>2020-06</t>
+          <t>2013-06</t>
         </is>
       </c>
       <c r="B139" t="n">
-        <v>0.0757</v>
-      </c>
-      <c r="C139" t="n">
-        <v>0.0186</v>
+        <v>0.004</v>
       </c>
     </row>
     <row r="140">
       <c r="A140" t="inlineStr">
         <is>
-          <t>2020-07</t>
+          <t>2013-07</t>
         </is>
       </c>
       <c r="B140" t="n">
-        <v>0.0424</v>
-      </c>
-      <c r="C140" t="n">
-        <v>0.0132</v>
+        <v>0.003</v>
       </c>
     </row>
     <row r="141">
       <c r="A141" t="inlineStr">
         <is>
-          <t>2020-08</t>
+          <t>2013-08</t>
         </is>
       </c>
       <c r="B141" t="n">
-        <v>0.0379</v>
-      </c>
-      <c r="C141" t="n">
-        <v>0.0126</v>
+        <v>0.0018</v>
       </c>
     </row>
     <row r="142">
       <c r="A142" t="inlineStr">
         <is>
-          <t>2020-09</t>
+          <t>2013-09</t>
         </is>
       </c>
       <c r="B142" t="n">
-        <v>0.0645</v>
-      </c>
-      <c r="C142" t="n">
-        <v>0.0182</v>
+        <v>0.0037</v>
       </c>
     </row>
     <row r="143">
       <c r="A143" t="inlineStr">
         <is>
-          <t>2020-10</t>
+          <t>2013-10</t>
         </is>
       </c>
       <c r="B143" t="n">
-        <v>0.1176</v>
-      </c>
-      <c r="C143" t="n">
-        <v>0.0446</v>
+        <v>0.0098</v>
       </c>
     </row>
     <row r="144">
       <c r="A144" t="inlineStr">
         <is>
-          <t>2020-11</t>
+          <t>2013-11</t>
         </is>
       </c>
       <c r="B144" t="n">
-        <v>0.0969</v>
-      </c>
-      <c r="C144" t="n">
-        <v>0.0499</v>
+        <v>0.0213</v>
       </c>
     </row>
     <row r="145">
       <c r="A145" t="inlineStr">
         <is>
-          <t>2020-12</t>
+          <t>2013-12</t>
         </is>
       </c>
       <c r="B145" t="n">
-        <v>0.1322</v>
-      </c>
-      <c r="C145" t="n">
-        <v>0.1053</v>
+        <v>0.0477</v>
       </c>
     </row>
     <row r="146">
       <c r="A146" t="inlineStr">
         <is>
-          <t>2021-01</t>
+          <t>2014-01</t>
         </is>
       </c>
       <c r="B146" t="n">
-        <v>0.1345</v>
-      </c>
-      <c r="C146" t="n">
-        <v>0.1044</v>
+        <v>0.0607</v>
       </c>
     </row>
     <row r="147">
       <c r="A147" t="inlineStr">
         <is>
-          <t>2021-02</t>
+          <t>2014-02</t>
         </is>
       </c>
       <c r="B147" t="n">
-        <v>0.0985</v>
-      </c>
-      <c r="C147" t="n">
-        <v>0.0634</v>
+        <v>0.0494</v>
       </c>
     </row>
     <row r="148">
       <c r="A148" t="inlineStr">
         <is>
-          <t>2021-03</t>
+          <t>2014-03</t>
         </is>
       </c>
       <c r="B148" t="n">
-        <v>0.1021</v>
-      </c>
-      <c r="C148" t="n">
-        <v>0.0366</v>
+        <v>0.0283</v>
       </c>
     </row>
     <row r="149">
       <c r="A149" t="inlineStr">
         <is>
-          <t>2021-04</t>
+          <t>2014-04</t>
         </is>
       </c>
       <c r="B149" t="n">
-        <v>0.063</v>
-      </c>
-      <c r="C149" t="n">
-        <v>0.0163</v>
+        <v>0.0127</v>
       </c>
     </row>
     <row r="150">
       <c r="A150" t="inlineStr">
         <is>
-          <t>2021-05</t>
+          <t>2014-05</t>
         </is>
       </c>
       <c r="B150" t="n">
-        <v>0.0561</v>
-      </c>
-      <c r="C150" t="n">
-        <v>0.0136</v>
+        <v>0.006</v>
       </c>
     </row>
     <row r="151">
       <c r="A151" t="inlineStr">
         <is>
-          <t>2021-06</t>
+          <t>2014-06</t>
         </is>
       </c>
       <c r="B151" t="n">
-        <v>0.0442</v>
-      </c>
-      <c r="C151" t="n">
-        <v>0.0101</v>
+        <v>0.004</v>
       </c>
     </row>
     <row r="152">
       <c r="A152" t="inlineStr">
         <is>
-          <t>2021-07</t>
+          <t>2014-07</t>
         </is>
       </c>
       <c r="B152" t="n">
-        <v>0.0504</v>
-      </c>
-      <c r="C152" t="n">
-        <v>0.0107</v>
+        <v>0.0027</v>
       </c>
     </row>
     <row r="153">
       <c r="A153" t="inlineStr">
         <is>
-          <t>2021-08</t>
+          <t>2014-08</t>
         </is>
       </c>
       <c r="B153" t="n">
-        <v>0.0519</v>
-      </c>
-      <c r="C153" t="n">
-        <v>0.0216</v>
+        <v>0.003</v>
       </c>
     </row>
     <row r="154">
       <c r="A154" t="inlineStr">
         <is>
-          <t>2021-09</t>
+          <t>2014-09</t>
         </is>
       </c>
       <c r="B154" t="n">
-        <v>0.0405</v>
-      </c>
-      <c r="C154" t="n">
-        <v>0.0124</v>
+        <v>0.0053</v>
       </c>
     </row>
     <row r="155">
       <c r="A155" t="inlineStr">
         <is>
-          <t>2021-10</t>
+          <t>2014-10</t>
         </is>
       </c>
       <c r="B155" t="n">
-        <v>0.1039</v>
-      </c>
-      <c r="C155" t="n">
-        <v>0.0348</v>
+        <v>0.0091</v>
       </c>
     </row>
     <row r="156">
       <c r="A156" t="inlineStr">
         <is>
-          <t>2021-11</t>
+          <t>2014-11</t>
         </is>
       </c>
       <c r="B156" t="n">
-        <v>0.1297</v>
-      </c>
-      <c r="C156" t="n">
-        <v>0.065</v>
+        <v>0.0239</v>
       </c>
     </row>
     <row r="157">
       <c r="A157" t="inlineStr">
         <is>
-          <t>2021-12</t>
+          <t>2014-12</t>
         </is>
       </c>
       <c r="B157" t="n">
-        <v>0.1638</v>
-      </c>
-      <c r="C157" t="n">
-        <v>0.1117</v>
+        <v>0.0448</v>
       </c>
     </row>
     <row r="158">
       <c r="A158" t="inlineStr">
         <is>
-          <t>2022-01</t>
+          <t>2015-01</t>
         </is>
       </c>
       <c r="B158" t="n">
-        <v>0.1466</v>
-      </c>
-      <c r="C158" t="n">
-        <v>0.1</v>
+        <v>0.0737</v>
       </c>
     </row>
     <row r="159">
       <c r="A159" t="inlineStr">
         <is>
-          <t>2022-02</t>
+          <t>2015-02</t>
         </is>
       </c>
       <c r="B159" t="n">
-        <v>0.1292</v>
-      </c>
-      <c r="C159" t="n">
-        <v>0.07729999999999999</v>
+        <v>0.0481</v>
       </c>
     </row>
     <row r="160">
       <c r="A160" t="inlineStr">
         <is>
-          <t>2022-03</t>
+          <t>2015-03</t>
         </is>
       </c>
       <c r="B160" t="n">
-        <v>0.0965</v>
-      </c>
-      <c r="C160" t="n">
-        <v>0.0333</v>
+        <v>0.0357</v>
       </c>
     </row>
     <row r="161">
       <c r="A161" t="inlineStr">
         <is>
-          <t>2022-04</t>
+          <t>2015-04</t>
         </is>
       </c>
       <c r="B161" t="n">
-        <v>0.08890000000000001</v>
-      </c>
-      <c r="C161" t="n">
-        <v>0.0227</v>
+        <v>0.0213</v>
       </c>
     </row>
     <row r="162">
       <c r="A162" t="inlineStr">
         <is>
-          <t>2022-05</t>
+          <t>2015-05</t>
         </is>
       </c>
       <c r="B162" t="n">
-        <v>0.0766</v>
-      </c>
-      <c r="C162" t="n">
-        <v>0.0119</v>
+        <v>0.0131</v>
       </c>
     </row>
     <row r="163">
       <c r="A163" t="inlineStr">
         <is>
-          <t>2022-06</t>
+          <t>2015-06</t>
         </is>
       </c>
       <c r="B163" t="n">
-        <v>0.0547</v>
-      </c>
-      <c r="C163" t="n">
-        <v>0.0106</v>
+        <v>0.0075</v>
       </c>
     </row>
     <row r="164">
       <c r="A164" t="inlineStr">
         <is>
-          <t>2022-07</t>
+          <t>2015-07</t>
         </is>
       </c>
       <c r="B164" t="n">
-        <v>0.0446</v>
-      </c>
-      <c r="C164" t="n">
-        <v>0.0101</v>
+        <v>0.0066</v>
       </c>
     </row>
     <row r="165">
       <c r="A165" t="inlineStr">
         <is>
-          <t>2022-08</t>
+          <t>2015-08</t>
         </is>
       </c>
       <c r="B165" t="n">
-        <v>0.042</v>
-      </c>
-      <c r="C165" t="n">
-        <v>0.009900000000000001</v>
+        <v>0.0052</v>
       </c>
     </row>
     <row r="166">
       <c r="A166" t="inlineStr">
         <is>
-          <t>2022-09</t>
+          <t>2015-09</t>
         </is>
       </c>
       <c r="B166" t="n">
-        <v>0.0717</v>
-      </c>
-      <c r="C166" t="n">
-        <v>0.0161</v>
+        <v>0.0059</v>
       </c>
     </row>
     <row r="167">
       <c r="A167" t="inlineStr">
         <is>
-          <t>2022-10</t>
+          <t>2015-10</t>
         </is>
       </c>
       <c r="B167" t="n">
-        <v>0.0946</v>
-      </c>
-      <c r="C167" t="n">
-        <v>0.0325</v>
+        <v>0.0197</v>
       </c>
     </row>
     <row r="168">
       <c r="A168" t="inlineStr">
         <is>
-          <t>2022-11</t>
+          <t>2015-11</t>
         </is>
       </c>
       <c r="B168" t="n">
-        <v>0.0969</v>
-      </c>
-      <c r="C168" t="n">
-        <v>0.0534</v>
+        <v>0.0623</v>
       </c>
     </row>
     <row r="169">
       <c r="A169" t="inlineStr">
         <is>
-          <t>2022-12</t>
+          <t>2015-12</t>
         </is>
       </c>
       <c r="B169" t="n">
-        <v>0.1258</v>
-      </c>
-      <c r="C169" t="n">
-        <v>0.1039</v>
+        <v>0.0848</v>
       </c>
     </row>
     <row r="170">
       <c r="A170" t="inlineStr">
         <is>
-          <t>2023-01</t>
+          <t>2016-01</t>
         </is>
       </c>
       <c r="B170" t="n">
-        <v>0.1328</v>
-      </c>
-      <c r="C170" t="n">
-        <v>0.109</v>
+        <v>0.1055</v>
       </c>
     </row>
     <row r="171">
       <c r="A171" t="inlineStr">
         <is>
-          <t>2023-02</t>
+          <t>2016-02</t>
         </is>
       </c>
       <c r="B171" t="n">
-        <v>0.1106</v>
-      </c>
-      <c r="C171" t="n">
-        <v>0.07969999999999999</v>
+        <v>0.1008</v>
       </c>
     </row>
     <row r="172">
       <c r="A172" t="inlineStr">
         <is>
-          <t>2023-03</t>
+          <t>2016-03</t>
         </is>
       </c>
       <c r="B172" t="n">
-        <v>0.0974</v>
-      </c>
-      <c r="C172" t="n">
-        <v>0.0352</v>
+        <v>0.0389</v>
       </c>
     </row>
     <row r="173">
       <c r="A173" t="inlineStr">
         <is>
-          <t>2023-04</t>
+          <t>2016-04</t>
         </is>
       </c>
       <c r="B173" t="n">
-        <v>0.07240000000000001</v>
-      </c>
-      <c r="C173" t="n">
-        <v>0.0187</v>
+        <v>0.0168</v>
       </c>
     </row>
     <row r="174">
       <c r="A174" t="inlineStr">
         <is>
-          <t>2023-05</t>
+          <t>2016-05</t>
         </is>
       </c>
       <c r="B174" t="n">
-        <v>0.0552</v>
-      </c>
-      <c r="C174" t="n">
-        <v>0.0101</v>
+        <v>0.009599999999999999</v>
       </c>
     </row>
     <row r="175">
       <c r="A175" t="inlineStr">
         <is>
-          <t>2023-06</t>
+          <t>2016-06</t>
         </is>
       </c>
       <c r="B175" t="n">
-        <v>0.059</v>
-      </c>
-      <c r="C175" t="n">
-        <v>0.01</v>
+        <v>0.0075</v>
       </c>
     </row>
     <row r="176">
       <c r="A176" t="inlineStr">
         <is>
-          <t>2023-07</t>
+          <t>2016-07</t>
         </is>
       </c>
       <c r="B176" t="n">
-        <v>0.0484</v>
-      </c>
-      <c r="C176" t="n">
-        <v>0.008200000000000001</v>
+        <v>0.0067</v>
       </c>
     </row>
     <row r="177">
       <c r="A177" t="inlineStr">
         <is>
-          <t>2023-08</t>
+          <t>2016-08</t>
         </is>
       </c>
       <c r="B177" t="n">
-        <v>0.0499</v>
-      </c>
-      <c r="C177" t="n">
-        <v>0.0074</v>
+        <v>0.0046</v>
       </c>
     </row>
     <row r="178">
       <c r="A178" t="inlineStr">
         <is>
-          <t>2023-09</t>
+          <t>2016-09</t>
         </is>
       </c>
       <c r="B178" t="n">
-        <v>0.0581</v>
-      </c>
-      <c r="C178" t="n">
-        <v>0.0114</v>
+        <v>0.0076</v>
       </c>
     </row>
     <row r="179">
       <c r="A179" t="inlineStr">
         <is>
-          <t>2023-10</t>
+          <t>2016-10</t>
         </is>
       </c>
       <c r="B179" t="n">
-        <v>0.1133</v>
-      </c>
-      <c r="C179" t="n">
-        <v>0.0246</v>
+        <v>0.0193</v>
       </c>
     </row>
     <row r="180">
       <c r="A180" t="inlineStr">
         <is>
-          <t>2023-11</t>
+          <t>2016-11</t>
         </is>
       </c>
       <c r="B180" t="n">
-        <v>0.0863</v>
-      </c>
-      <c r="C180" t="n">
-        <v>0.0595</v>
+        <v>0.05</v>
       </c>
     </row>
     <row r="181">
       <c r="A181" t="inlineStr">
         <is>
-          <t>2023-12</t>
+          <t>2016-12</t>
         </is>
       </c>
       <c r="B181" t="n">
-        <v>0.1071</v>
-      </c>
-      <c r="C181" t="n">
-        <v>0.09950000000000001</v>
+        <v>0.07439999999999999</v>
       </c>
     </row>
     <row r="182">
       <c r="A182" t="inlineStr">
         <is>
-          <t>2024-01</t>
+          <t>2017-01</t>
         </is>
       </c>
       <c r="B182" t="n">
-        <v>0.1191</v>
-      </c>
-      <c r="C182" t="n">
-        <v>0.1148</v>
+        <v>0.0759</v>
       </c>
     </row>
     <row r="183">
       <c r="A183" t="inlineStr">
         <is>
-          <t>2024-02</t>
+          <t>2017-02</t>
         </is>
       </c>
       <c r="B183" t="n">
-        <v>0.0964</v>
-      </c>
-      <c r="C183" t="n">
-        <v>0.08169999999999999</v>
+        <v>0.0566</v>
       </c>
     </row>
     <row r="184">
       <c r="A184" t="inlineStr">
         <is>
-          <t>2024-03</t>
+          <t>2017-03</t>
         </is>
       </c>
       <c r="B184" t="n">
-        <v>0.0673</v>
-      </c>
-      <c r="C184" t="n">
-        <v>0.0383</v>
+        <v>0.0266</v>
       </c>
     </row>
     <row r="185">
       <c r="A185" t="inlineStr">
         <is>
-          <t>2024-04</t>
+          <t>2017-04</t>
         </is>
       </c>
       <c r="B185" t="n">
-        <v>0.082</v>
-      </c>
-      <c r="C185" t="n">
-        <v>0.0224</v>
+        <v>0.0169</v>
       </c>
     </row>
     <row r="186">
       <c r="A186" t="inlineStr">
         <is>
-          <t>2024-05</t>
+          <t>2017-05</t>
         </is>
       </c>
       <c r="B186" t="n">
-        <v>0.06660000000000001</v>
-      </c>
-      <c r="C186" t="n">
-        <v>0.0129</v>
+        <v>0.0098</v>
       </c>
     </row>
     <row r="187">
       <c r="A187" t="inlineStr">
         <is>
-          <t>2024-06</t>
+          <t>2017-06</t>
         </is>
       </c>
       <c r="B187" t="n">
-        <v>0.0513</v>
-      </c>
-      <c r="C187" t="n">
-        <v>0.0121</v>
+        <v>0.0059</v>
       </c>
     </row>
     <row r="188">
       <c r="A188" t="inlineStr">
         <is>
-          <t>2024-07</t>
+          <t>2017-07</t>
         </is>
       </c>
       <c r="B188" t="n">
-        <v>0.0555</v>
-      </c>
-      <c r="C188" t="n">
-        <v>0.015</v>
+        <v>0.0033</v>
       </c>
     </row>
     <row r="189">
       <c r="A189" t="inlineStr">
         <is>
-          <t>2024-08</t>
+          <t>2017-08</t>
         </is>
       </c>
       <c r="B189" t="n">
-        <v>0.0482</v>
-      </c>
-      <c r="C189" t="n">
-        <v>0.0101</v>
+        <v>0.0047</v>
       </c>
     </row>
     <row r="190">
       <c r="A190" t="inlineStr">
         <is>
-          <t>2024-09</t>
+          <t>2017-09</t>
         </is>
       </c>
       <c r="B190" t="n">
-        <v>0.0672</v>
-      </c>
-      <c r="C190" t="n">
-        <v>0.0122</v>
+        <v>0.0051</v>
       </c>
     </row>
     <row r="191">
       <c r="A191" t="inlineStr">
         <is>
-          <t>2024-10</t>
+          <t>2017-10</t>
         </is>
       </c>
       <c r="B191" t="n">
-        <v>0.0921</v>
-      </c>
-      <c r="C191" t="n">
-        <v>0.0278</v>
+        <v>0.0158</v>
       </c>
     </row>
     <row r="192">
       <c r="A192" t="inlineStr">
         <is>
-          <t>2024-11</t>
+          <t>2017-11</t>
         </is>
       </c>
       <c r="B192" t="n">
-        <v>0.1151</v>
-      </c>
-      <c r="C192" t="n">
-        <v>0.0414</v>
+        <v>0.0256</v>
       </c>
     </row>
     <row r="193">
       <c r="A193" t="inlineStr">
         <is>
-          <t>2024-12</t>
+          <t>2017-12</t>
         </is>
       </c>
       <c r="B193" t="n">
-        <v>0.1316</v>
-      </c>
-      <c r="C193" t="n">
-        <v>0.1016</v>
+        <v>0.0426</v>
       </c>
     </row>
     <row r="194">
       <c r="A194" t="inlineStr">
         <is>
-          <t>2025-01</t>
+          <t>2018-01</t>
         </is>
       </c>
       <c r="B194" t="n">
-        <v>0.1362</v>
-      </c>
-      <c r="C194" t="n">
-        <v>0.09719999999999999</v>
+        <v>0.0425</v>
       </c>
     </row>
     <row r="195">
       <c r="A195" t="inlineStr">
         <is>
-          <t>2025-02</t>
+          <t>2018-02</t>
         </is>
       </c>
       <c r="B195" t="n">
-        <v>0.1154</v>
-      </c>
-      <c r="C195" t="n">
-        <v>0.0673</v>
+        <v>0.0364</v>
       </c>
     </row>
     <row r="196">
       <c r="A196" t="inlineStr">
         <is>
-          <t>2025-03</t>
+          <t>2018-03</t>
         </is>
       </c>
       <c r="B196" t="n">
-        <v>0.0815</v>
-      </c>
-      <c r="C196" t="n">
-        <v>0.0293</v>
+        <v>0.025</v>
       </c>
     </row>
     <row r="197">
       <c r="A197" t="inlineStr">
         <is>
-          <t>2025-04</t>
+          <t>2018-04</t>
         </is>
       </c>
       <c r="B197" t="n">
-        <v>0.0978</v>
-      </c>
-      <c r="C197" t="n">
-        <v>0.0201</v>
+        <v>0.0109</v>
       </c>
     </row>
     <row r="198">
       <c r="A198" t="inlineStr">
         <is>
-          <t>2025-05</t>
+          <t>2018-05</t>
         </is>
       </c>
       <c r="B198" t="n">
-        <v>0.0718</v>
-      </c>
-      <c r="C198" t="n">
-        <v>0.0139</v>
+        <v>0.0071</v>
       </c>
     </row>
     <row r="199">
       <c r="A199" t="inlineStr">
         <is>
-          <t>2025-06</t>
+          <t>2018-06</t>
         </is>
       </c>
       <c r="B199" t="n">
-        <v>0.0658</v>
-      </c>
-      <c r="C199" t="n">
-        <v>0.0157</v>
+        <v>0.0045</v>
       </c>
     </row>
     <row r="200">
       <c r="A200" t="inlineStr">
         <is>
-          <t>2025-07</t>
+          <t>2018-07</t>
         </is>
       </c>
       <c r="B200" t="n">
-        <v>0.0482</v>
-      </c>
-      <c r="C200" t="n">
-        <v>0.0105</v>
+        <v>0.0034</v>
       </c>
     </row>
     <row r="201">
       <c r="A201" t="inlineStr">
         <is>
-          <t>2025-08</t>
+          <t>2018-08</t>
         </is>
       </c>
       <c r="B201" t="n">
-        <v>0.0482</v>
-      </c>
-      <c r="C201" t="n">
-        <v>0.0095</v>
+        <v>0.0034</v>
       </c>
     </row>
     <row r="202">
       <c r="A202" t="inlineStr">
         <is>
-          <t>2025-09</t>
+          <t>2018-09</t>
         </is>
       </c>
       <c r="B202" t="n">
-        <v>0.0851</v>
-      </c>
-      <c r="C202" t="n">
-        <v>0.0138</v>
+        <v>0.0054</v>
       </c>
     </row>
     <row r="203">
       <c r="A203" t="inlineStr">
         <is>
-          <t>2025-10</t>
+          <t>2018-10</t>
         </is>
       </c>
       <c r="B203" t="n">
-        <v>0.09320000000000001</v>
-      </c>
-      <c r="C203" t="n">
-        <v>0.0263</v>
+        <v>0.0141</v>
       </c>
     </row>
     <row r="204">
       <c r="A204" t="inlineStr">
         <is>
-          <t>2025-11</t>
+          <t>2018-11</t>
         </is>
       </c>
       <c r="B204" t="n">
-        <v>0.1021</v>
-      </c>
-      <c r="C204" t="n">
-        <v>0.0486</v>
+        <v>0.0353</v>
       </c>
     </row>
     <row r="205">
       <c r="A205" t="inlineStr">
         <is>
-          <t>2025-12</t>
+          <t>2018-12</t>
         </is>
       </c>
       <c r="B205" t="n">
-        <v>0.0998</v>
-      </c>
-      <c r="C205" t="n">
-        <v>0.0735</v>
+        <v>0.0568</v>
       </c>
     </row>
     <row r="206">
       <c r="A206" t="inlineStr">
         <is>
-          <t>2026-01</t>
+          <t>2019-01</t>
         </is>
       </c>
       <c r="B206" t="n">
-        <v>0.08699999999999999</v>
-      </c>
-      <c r="C206" t="n">
-        <v>0.0677</v>
+        <v>0.06</v>
       </c>
     </row>
     <row r="207">
       <c r="A207" t="inlineStr">
         <is>
+          <t>2019-02</t>
+        </is>
+      </c>
+      <c r="B207" t="n">
+        <v>0.0477</v>
+      </c>
+    </row>
+    <row r="208">
+      <c r="A208" t="inlineStr">
+        <is>
+          <t>2019-03</t>
+        </is>
+      </c>
+      <c r="B208" t="n">
+        <v>0.0278</v>
+      </c>
+    </row>
+    <row r="209">
+      <c r="A209" t="inlineStr">
+        <is>
+          <t>2019-04</t>
+        </is>
+      </c>
+      <c r="B209" t="n">
+        <v>0.0175</v>
+      </c>
+    </row>
+    <row r="210">
+      <c r="A210" t="inlineStr">
+        <is>
+          <t>2019-05</t>
+        </is>
+      </c>
+      <c r="B210" t="n">
+        <v>0.0107</v>
+      </c>
+    </row>
+    <row r="211">
+      <c r="A211" t="inlineStr">
+        <is>
+          <t>2019-06</t>
+        </is>
+      </c>
+      <c r="B211" t="n">
+        <v>0.0095</v>
+      </c>
+    </row>
+    <row r="212">
+      <c r="A212" t="inlineStr">
+        <is>
+          <t>2019-07</t>
+        </is>
+      </c>
+      <c r="B212" t="n">
+        <v>0.006</v>
+      </c>
+    </row>
+    <row r="213">
+      <c r="A213" t="inlineStr">
+        <is>
+          <t>2019-08</t>
+        </is>
+      </c>
+      <c r="B213" t="n">
+        <v>0.007900000000000001</v>
+      </c>
+    </row>
+    <row r="214">
+      <c r="A214" t="inlineStr">
+        <is>
+          <t>2019-09</t>
+        </is>
+      </c>
+      <c r="B214" t="n">
+        <v>0.0106</v>
+      </c>
+    </row>
+    <row r="215">
+      <c r="A215" t="inlineStr">
+        <is>
+          <t>2019-10</t>
+        </is>
+      </c>
+      <c r="B215" t="n">
+        <v>0.0262</v>
+      </c>
+    </row>
+    <row r="216">
+      <c r="A216" t="inlineStr">
+        <is>
+          <t>2019-11</t>
+        </is>
+      </c>
+      <c r="B216" t="n">
+        <v>0.0611</v>
+      </c>
+    </row>
+    <row r="217">
+      <c r="A217" t="inlineStr">
+        <is>
+          <t>2019-12</t>
+        </is>
+      </c>
+      <c r="B217" t="n">
+        <v>0.106</v>
+      </c>
+    </row>
+    <row r="218">
+      <c r="A218" t="inlineStr">
+        <is>
+          <t>2020-01</t>
+        </is>
+      </c>
+      <c r="B218" t="n">
+        <v>0.1203</v>
+      </c>
+    </row>
+    <row r="219">
+      <c r="A219" t="inlineStr">
+        <is>
+          <t>2020-02</t>
+        </is>
+      </c>
+      <c r="B219" t="n">
+        <v>0.07679999999999999</v>
+      </c>
+    </row>
+    <row r="220">
+      <c r="A220" t="inlineStr">
+        <is>
+          <t>2020-03</t>
+        </is>
+      </c>
+      <c r="B220" t="n">
+        <v>0.04</v>
+      </c>
+    </row>
+    <row r="221">
+      <c r="A221" t="inlineStr">
+        <is>
+          <t>2020-04</t>
+        </is>
+      </c>
+      <c r="B221" t="n">
+        <v>0.0224</v>
+      </c>
+    </row>
+    <row r="222">
+      <c r="A222" t="inlineStr">
+        <is>
+          <t>2020-05</t>
+        </is>
+      </c>
+      <c r="B222" t="n">
+        <v>0.0089</v>
+      </c>
+    </row>
+    <row r="223">
+      <c r="A223" t="inlineStr">
+        <is>
+          <t>2020-06</t>
+        </is>
+      </c>
+      <c r="B223" t="n">
+        <v>0.0058</v>
+      </c>
+    </row>
+    <row r="224">
+      <c r="A224" t="inlineStr">
+        <is>
+          <t>2020-07</t>
+        </is>
+      </c>
+      <c r="B224" t="n">
+        <v>0.0036</v>
+      </c>
+    </row>
+    <row r="225">
+      <c r="A225" t="inlineStr">
+        <is>
+          <t>2020-08</t>
+        </is>
+      </c>
+      <c r="B225" t="n">
+        <v>0.0037</v>
+      </c>
+    </row>
+    <row r="226">
+      <c r="A226" t="inlineStr">
+        <is>
+          <t>2020-09</t>
+        </is>
+      </c>
+      <c r="B226" t="n">
+        <v>0.008699999999999999</v>
+      </c>
+    </row>
+    <row r="227">
+      <c r="A227" t="inlineStr">
+        <is>
+          <t>2020-10</t>
+        </is>
+      </c>
+      <c r="B227" t="n">
+        <v>0.031</v>
+      </c>
+    </row>
+    <row r="228">
+      <c r="A228" t="inlineStr">
+        <is>
+          <t>2020-11</t>
+        </is>
+      </c>
+      <c r="B228" t="n">
+        <v>0.0767</v>
+      </c>
+    </row>
+    <row r="229">
+      <c r="A229" t="inlineStr">
+        <is>
+          <t>2020-12</t>
+        </is>
+      </c>
+      <c r="B229" t="n">
+        <v>0.2106</v>
+      </c>
+    </row>
+    <row r="230">
+      <c r="A230" t="inlineStr">
+        <is>
+          <t>2021-01</t>
+        </is>
+      </c>
+      <c r="B230" t="n">
+        <v>0.2158</v>
+      </c>
+    </row>
+    <row r="231">
+      <c r="A231" t="inlineStr">
+        <is>
+          <t>2021-02</t>
+        </is>
+      </c>
+      <c r="B231" t="n">
+        <v>0.1389</v>
+      </c>
+    </row>
+    <row r="232">
+      <c r="A232" t="inlineStr">
+        <is>
+          <t>2021-03</t>
+        </is>
+      </c>
+      <c r="B232" t="n">
+        <v>0.0626</v>
+      </c>
+    </row>
+    <row r="233">
+      <c r="A233" t="inlineStr">
+        <is>
+          <t>2021-04</t>
+        </is>
+      </c>
+      <c r="B233" t="n">
+        <v>0.0363</v>
+      </c>
+    </row>
+    <row r="234">
+      <c r="A234" t="inlineStr">
+        <is>
+          <t>2021-05</t>
+        </is>
+      </c>
+      <c r="B234" t="n">
+        <v>0.0195</v>
+      </c>
+    </row>
+    <row r="235">
+      <c r="A235" t="inlineStr">
+        <is>
+          <t>2021-06</t>
+        </is>
+      </c>
+      <c r="B235" t="n">
+        <v>0.0106</v>
+      </c>
+    </row>
+    <row r="236">
+      <c r="A236" t="inlineStr">
+        <is>
+          <t>2021-07</t>
+        </is>
+      </c>
+      <c r="B236" t="n">
+        <v>0.0118</v>
+      </c>
+    </row>
+    <row r="237">
+      <c r="A237" t="inlineStr">
+        <is>
+          <t>2021-08</t>
+        </is>
+      </c>
+      <c r="B237" t="n">
+        <v>0.009299999999999999</v>
+      </c>
+    </row>
+    <row r="238">
+      <c r="A238" t="inlineStr">
+        <is>
+          <t>2021-09</t>
+        </is>
+      </c>
+      <c r="B238" t="n">
+        <v>0.0113</v>
+      </c>
+    </row>
+    <row r="239">
+      <c r="A239" t="inlineStr">
+        <is>
+          <t>2021-10</t>
+        </is>
+      </c>
+      <c r="B239" t="n">
+        <v>0.0409</v>
+      </c>
+    </row>
+    <row r="240">
+      <c r="A240" t="inlineStr">
+        <is>
+          <t>2021-11</t>
+        </is>
+      </c>
+      <c r="B240" t="n">
+        <v>0.0922</v>
+      </c>
+    </row>
+    <row r="241">
+      <c r="A241" t="inlineStr">
+        <is>
+          <t>2021-12</t>
+        </is>
+      </c>
+      <c r="B241" t="n">
+        <v>0.142</v>
+      </c>
+    </row>
+    <row r="242">
+      <c r="A242" t="inlineStr">
+        <is>
+          <t>2022-01</t>
+        </is>
+      </c>
+      <c r="B242" t="n">
+        <v>0.1604</v>
+      </c>
+    </row>
+    <row r="243">
+      <c r="A243" t="inlineStr">
+        <is>
+          <t>2022-02</t>
+        </is>
+      </c>
+      <c r="B243" t="n">
+        <v>0.1286</v>
+      </c>
+    </row>
+    <row r="244">
+      <c r="A244" t="inlineStr">
+        <is>
+          <t>2022-03</t>
+        </is>
+      </c>
+      <c r="B244" t="n">
+        <v>0.07729999999999999</v>
+      </c>
+    </row>
+    <row r="245">
+      <c r="A245" t="inlineStr">
+        <is>
+          <t>2022-04</t>
+        </is>
+      </c>
+      <c r="B245" t="n">
+        <v>0.052</v>
+      </c>
+    </row>
+    <row r="246">
+      <c r="A246" t="inlineStr">
+        <is>
+          <t>2022-05</t>
+        </is>
+      </c>
+      <c r="B246" t="n">
+        <v>0.0177</v>
+      </c>
+    </row>
+    <row r="247">
+      <c r="A247" t="inlineStr">
+        <is>
+          <t>2022-06</t>
+        </is>
+      </c>
+      <c r="B247" t="n">
+        <v>0.0103</v>
+      </c>
+    </row>
+    <row r="248">
+      <c r="A248" t="inlineStr">
+        <is>
+          <t>2022-07</t>
+        </is>
+      </c>
+      <c r="B248" t="n">
+        <v>0.0074</v>
+      </c>
+    </row>
+    <row r="249">
+      <c r="A249" t="inlineStr">
+        <is>
+          <t>2022-08</t>
+        </is>
+      </c>
+      <c r="B249" t="n">
+        <v>0.0064</v>
+      </c>
+    </row>
+    <row r="250">
+      <c r="A250" t="inlineStr">
+        <is>
+          <t>2022-09</t>
+        </is>
+      </c>
+      <c r="B250" t="n">
+        <v>0.013</v>
+      </c>
+    </row>
+    <row r="251">
+      <c r="A251" t="inlineStr">
+        <is>
+          <t>2022-10</t>
+        </is>
+      </c>
+      <c r="B251" t="n">
+        <v>0.0483</v>
+      </c>
+    </row>
+    <row r="252">
+      <c r="A252" t="inlineStr">
+        <is>
+          <t>2022-11</t>
+        </is>
+      </c>
+      <c r="B252" t="n">
+        <v>0.0834</v>
+      </c>
+    </row>
+    <row r="253">
+      <c r="A253" t="inlineStr">
+        <is>
+          <t>2022-12</t>
+        </is>
+      </c>
+      <c r="B253" t="n">
+        <v>0.1377</v>
+      </c>
+    </row>
+    <row r="254">
+      <c r="A254" t="inlineStr">
+        <is>
+          <t>2023-01</t>
+        </is>
+      </c>
+      <c r="B254" t="n">
+        <v>0.1632</v>
+      </c>
+    </row>
+    <row r="255">
+      <c r="A255" t="inlineStr">
+        <is>
+          <t>2023-02</t>
+        </is>
+      </c>
+      <c r="B255" t="n">
+        <v>0.1098</v>
+      </c>
+    </row>
+    <row r="256">
+      <c r="A256" t="inlineStr">
+        <is>
+          <t>2023-03</t>
+        </is>
+      </c>
+      <c r="B256" t="n">
+        <v>0.0514</v>
+      </c>
+    </row>
+    <row r="257">
+      <c r="A257" t="inlineStr">
+        <is>
+          <t>2023-04</t>
+        </is>
+      </c>
+      <c r="B257" t="n">
+        <v>0.029</v>
+      </c>
+    </row>
+    <row r="258">
+      <c r="A258" t="inlineStr">
+        <is>
+          <t>2023-05</t>
+        </is>
+      </c>
+      <c r="B258" t="n">
+        <v>0.016</v>
+      </c>
+    </row>
+    <row r="259">
+      <c r="A259" t="inlineStr">
+        <is>
+          <t>2023-06</t>
+        </is>
+      </c>
+      <c r="B259" t="n">
+        <v>0.0117</v>
+      </c>
+    </row>
+    <row r="260">
+      <c r="A260" t="inlineStr">
+        <is>
+          <t>2023-07</t>
+        </is>
+      </c>
+      <c r="B260" t="n">
+        <v>0.0116</v>
+      </c>
+    </row>
+    <row r="261">
+      <c r="A261" t="inlineStr">
+        <is>
+          <t>2023-08</t>
+        </is>
+      </c>
+      <c r="B261" t="n">
+        <v>0.0057</v>
+      </c>
+    </row>
+    <row r="262">
+      <c r="A262" t="inlineStr">
+        <is>
+          <t>2023-09</t>
+        </is>
+      </c>
+      <c r="B262" t="n">
+        <v>0.007900000000000001</v>
+      </c>
+    </row>
+    <row r="263">
+      <c r="A263" t="inlineStr">
+        <is>
+          <t>2023-10</t>
+        </is>
+      </c>
+      <c r="B263" t="n">
+        <v>0.0245</v>
+      </c>
+    </row>
+    <row r="264">
+      <c r="A264" t="inlineStr">
+        <is>
+          <t>2023-11</t>
+        </is>
+      </c>
+      <c r="B264" t="n">
+        <v>0.0576</v>
+      </c>
+    </row>
+    <row r="265">
+      <c r="A265" t="inlineStr">
+        <is>
+          <t>2023-12</t>
+        </is>
+      </c>
+      <c r="B265" t="n">
+        <v>0.1155</v>
+      </c>
+    </row>
+    <row r="266">
+      <c r="A266" t="inlineStr">
+        <is>
+          <t>2024-01</t>
+        </is>
+      </c>
+      <c r="B266" t="n">
+        <v>0.1383</v>
+      </c>
+    </row>
+    <row r="267">
+      <c r="A267" t="inlineStr">
+        <is>
+          <t>2024-02</t>
+        </is>
+      </c>
+      <c r="B267" t="n">
+        <v>0.1074</v>
+      </c>
+    </row>
+    <row r="268">
+      <c r="A268" t="inlineStr">
+        <is>
+          <t>2024-03</t>
+        </is>
+      </c>
+      <c r="B268" t="n">
+        <v>0.0568</v>
+      </c>
+    </row>
+    <row r="269">
+      <c r="A269" t="inlineStr">
+        <is>
+          <t>2024-04</t>
+        </is>
+      </c>
+      <c r="B269" t="n">
+        <v>0.0247</v>
+      </c>
+    </row>
+    <row r="270">
+      <c r="A270" t="inlineStr">
+        <is>
+          <t>2024-05</t>
+        </is>
+      </c>
+      <c r="B270" t="n">
+        <v>0.0168</v>
+      </c>
+    </row>
+    <row r="271">
+      <c r="A271" t="inlineStr">
+        <is>
+          <t>2024-06</t>
+        </is>
+      </c>
+      <c r="B271" t="n">
+        <v>0.007900000000000001</v>
+      </c>
+    </row>
+    <row r="272">
+      <c r="A272" t="inlineStr">
+        <is>
+          <t>2024-07</t>
+        </is>
+      </c>
+      <c r="B272" t="n">
+        <v>0.0078</v>
+      </c>
+    </row>
+    <row r="273">
+      <c r="A273" t="inlineStr">
+        <is>
+          <t>2024-08</t>
+        </is>
+      </c>
+      <c r="B273" t="n">
+        <v>0.0056</v>
+      </c>
+    </row>
+    <row r="274">
+      <c r="A274" t="inlineStr">
+        <is>
+          <t>2024-09</t>
+        </is>
+      </c>
+      <c r="B274" t="n">
+        <v>0.01</v>
+      </c>
+    </row>
+    <row r="275">
+      <c r="A275" t="inlineStr">
+        <is>
+          <t>2024-10</t>
+        </is>
+      </c>
+      <c r="B275" t="n">
+        <v>0.036</v>
+      </c>
+    </row>
+    <row r="276">
+      <c r="A276" t="inlineStr">
+        <is>
+          <t>2024-11</t>
+        </is>
+      </c>
+      <c r="B276" t="n">
+        <v>0.053</v>
+      </c>
+    </row>
+    <row r="277">
+      <c r="A277" t="inlineStr">
+        <is>
+          <t>2024-12</t>
+        </is>
+      </c>
+      <c r="B277" t="n">
+        <v>0.122</v>
+      </c>
+    </row>
+    <row r="278">
+      <c r="A278" t="inlineStr">
+        <is>
+          <t>2025-01</t>
+        </is>
+      </c>
+      <c r="B278" t="n">
+        <v>0.1336</v>
+      </c>
+    </row>
+    <row r="279">
+      <c r="A279" t="inlineStr">
+        <is>
+          <t>2025-02</t>
+        </is>
+      </c>
+      <c r="B279" t="n">
+        <v>0.08210000000000001</v>
+      </c>
+    </row>
+    <row r="280">
+      <c r="A280" t="inlineStr">
+        <is>
+          <t>2025-03</t>
+        </is>
+      </c>
+      <c r="B280" t="n">
+        <v>0.0356</v>
+      </c>
+    </row>
+    <row r="281">
+      <c r="A281" t="inlineStr">
+        <is>
+          <t>2025-04</t>
+        </is>
+      </c>
+      <c r="B281" t="n">
+        <v>0.0229</v>
+      </c>
+    </row>
+    <row r="282">
+      <c r="A282" t="inlineStr">
+        <is>
+          <t>2025-05</t>
+        </is>
+      </c>
+      <c r="B282" t="n">
+        <v>0.0117</v>
+      </c>
+    </row>
+    <row r="283">
+      <c r="A283" t="inlineStr">
+        <is>
+          <t>2025-06</t>
+        </is>
+      </c>
+      <c r="B283" t="n">
+        <v>0.008399999999999999</v>
+      </c>
+    </row>
+    <row r="284">
+      <c r="A284" t="inlineStr">
+        <is>
+          <t>2025-07</t>
+        </is>
+      </c>
+      <c r="B284" t="n">
+        <v>0.0058</v>
+      </c>
+    </row>
+    <row r="285">
+      <c r="A285" t="inlineStr">
+        <is>
+          <t>2025-08</t>
+        </is>
+      </c>
+      <c r="B285" t="n">
+        <v>0.0057</v>
+      </c>
+    </row>
+    <row r="286">
+      <c r="A286" t="inlineStr">
+        <is>
+          <t>2025-09</t>
+        </is>
+      </c>
+      <c r="B286" t="n">
+        <v>0.0089</v>
+      </c>
+    </row>
+    <row r="287">
+      <c r="A287" t="inlineStr">
+        <is>
+          <t>2025-10</t>
+        </is>
+      </c>
+      <c r="B287" t="n">
+        <v>0.0211</v>
+      </c>
+    </row>
+    <row r="288">
+      <c r="A288" t="inlineStr">
+        <is>
+          <t>2025-11</t>
+        </is>
+      </c>
+      <c r="B288" t="n">
+        <v>0.0293</v>
+      </c>
+    </row>
+    <row r="289">
+      <c r="A289" t="inlineStr">
+        <is>
+          <t>2025-12</t>
+        </is>
+      </c>
+      <c r="B289" t="n">
+        <v>0.0438</v>
+      </c>
+    </row>
+    <row r="290">
+      <c r="A290" t="inlineStr">
+        <is>
+          <t>2026-01</t>
+        </is>
+      </c>
+      <c r="B290" t="n">
+        <v>0.048</v>
+      </c>
+    </row>
+    <row r="291">
+      <c r="A291" t="inlineStr">
+        <is>
           <t>2026-02</t>
         </is>
       </c>
-      <c r="B207" t="n">
-        <v>0.08110000000000001</v>
-      </c>
-      <c r="C207" t="n">
-        <v>0.0469</v>
+      <c r="B291" t="n">
+        <v>0.0334</v>
+      </c>
+    </row>
+    <row r="292">
+      <c r="A292" t="inlineStr">
+        <is>
+          <t>2026-03</t>
+        </is>
+      </c>
+      <c r="B292" t="n">
+        <v>0.0208</v>
+      </c>
+    </row>
+    <row r="293">
+      <c r="A293" t="inlineStr">
+        <is>
+          <t>2026-04</t>
+        </is>
+      </c>
+      <c r="B293" t="n">
+        <v>0.0135</v>
+      </c>
+    </row>
+    <row r="294">
+      <c r="A294" t="inlineStr">
+        <is>
+          <t>2026-05</t>
+        </is>
+      </c>
+      <c r="B294" t="n">
+        <v>0.008699999999999999</v>
+      </c>
+    </row>
+    <row r="295">
+      <c r="A295" t="inlineStr">
+        <is>
+          <t>2026-06</t>
+        </is>
+      </c>
+      <c r="B295" t="n">
+        <v>0.0056</v>
+      </c>
+    </row>
+    <row r="296">
+      <c r="A296" t="inlineStr">
+        <is>
+          <t>2026-07</t>
+        </is>
+      </c>
+      <c r="B296" t="n">
+        <v>0.0041</v>
+      </c>
+    </row>
+    <row r="297">
+      <c r="A297" t="inlineStr">
+        <is>
+          <t>2026-08</t>
+        </is>
+      </c>
+      <c r="B297" t="n">
+        <v>0.0034</v>
       </c>
     </row>
   </sheetData>

</xml_diff>